<commit_message>
fix: actualizar.py resuelve nombres KO via bracket_manuales; pipeline más robusto; deploy cada hora
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Mundial2026_Tracker.xlsx
+++ b/output/Mundial2026_Tracker.xlsx
@@ -7598,9 +7598,17 @@
       <c r="A74" s="2" t="n">
         <v>73</v>
       </c>
-      <c r="B74" s="3" t="n"/>
-      <c r="C74" s="3" t="n"/>
-      <c r="D74" s="3" t="n"/>
+      <c r="B74" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C74" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="E74" s="3" t="n"/>
       <c r="F74" s="2">
         <f>VLOOKUP($A74,Fixture!$A:$F,5,0)</f>
@@ -7615,9 +7623,17 @@
       <c r="A75" s="2" t="n">
         <v>74</v>
       </c>
-      <c r="B75" s="3" t="n"/>
-      <c r="C75" s="3" t="n"/>
-      <c r="D75" s="3" t="n"/>
+      <c r="B75" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="E75" s="3" t="n"/>
       <c r="F75" s="2">
         <f>VLOOKUP($A75,Fixture!$A:$F,5,0)</f>
@@ -7632,43 +7648,71 @@
       <c r="A76" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="B76" s="3" t="n"/>
-      <c r="C76" s="3" t="n"/>
-      <c r="D76" s="3" t="n"/>
-      <c r="E76" s="3" t="n"/>
-      <c r="F76" s="2">
-        <f>VLOOKUP($A76,Fixture!$A:$F,5,0)</f>
-        <v/>
-      </c>
-      <c r="G76" s="2">
-        <f>VLOOKUP($A76,Fixture!$A:$F,6,0)</f>
-        <v/>
+      <c r="B76" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="G76" s="2" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="2" t="n">
         <v>76</v>
       </c>
-      <c r="B77" s="3" t="n"/>
-      <c r="C77" s="3" t="n"/>
-      <c r="D77" s="3" t="n"/>
-      <c r="E77" s="3" t="n"/>
-      <c r="F77" s="2">
-        <f>VLOOKUP($A77,Fixture!$A:$F,5,0)</f>
-        <v/>
-      </c>
-      <c r="G77" s="2">
-        <f>VLOOKUP($A77,Fixture!$A:$F,6,0)</f>
-        <v/>
+      <c r="B77" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>Marruecos</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G77" s="2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1">
       <c r="A78" s="2" t="n">
         <v>77</v>
       </c>
-      <c r="B78" s="3" t="n"/>
-      <c r="C78" s="3" t="n"/>
-      <c r="D78" s="3" t="n"/>
+      <c r="B78" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="E78" s="3" t="n"/>
       <c r="F78" s="2">
         <f>VLOOKUP($A78,Fixture!$A:$F,5,0)</f>

</xml_diff>

<commit_message>
fix: cargar resultados de Octavos y corregir bracket_manuales
- Agrega overrides en bracket_manuales.json para partidos de Octavos
  (IDs 89, 91, 95, 96) donde el bracket real del Mundial difiere del
  pre-seeding cargado en el Fixture
- Agrega ±1 día de tolerancia en búsqueda ESPN vs Fixture para cubrir
  diferencias horarias de hasta 1 día en ambas direcciones
- Agrega nombres ESPN faltantes a ESPN_EXTRA (Canada, France, Egypt...)
- Carga 7/8 resultados de Octavos en el xlsx; ID 96 pendiente (hoy)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/Mundial2026_Tracker.xlsx
+++ b/output/Mundial2026_Tracker.xlsx
@@ -8004,9 +8004,17 @@
       <c r="A90" s="2" t="n">
         <v>89</v>
       </c>
-      <c r="B90" s="3" t="n"/>
-      <c r="C90" s="3" t="n"/>
-      <c r="D90" s="3" t="n"/>
+      <c r="B90" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C90" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="E90" s="3" t="n"/>
       <c r="F90" s="2">
         <f>VLOOKUP($A90,Fixture!$A:$F,5,0)</f>
@@ -8021,9 +8029,17 @@
       <c r="A91" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="B91" s="3" t="n"/>
-      <c r="C91" s="3" t="n"/>
-      <c r="D91" s="3" t="n"/>
+      <c r="B91" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C91" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="E91" s="3" t="n"/>
       <c r="F91" s="2">
         <f>VLOOKUP($A91,Fixture!$A:$F,5,0)</f>
@@ -8038,9 +8054,17 @@
       <c r="A92" s="2" t="n">
         <v>91</v>
       </c>
-      <c r="B92" s="3" t="n"/>
-      <c r="C92" s="3" t="n"/>
-      <c r="D92" s="3" t="n"/>
+      <c r="B92" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="E92" s="3" t="n"/>
       <c r="F92" s="2">
         <f>VLOOKUP($A92,Fixture!$A:$F,5,0)</f>
@@ -8055,9 +8079,17 @@
       <c r="A93" s="2" t="n">
         <v>92</v>
       </c>
-      <c r="B93" s="3" t="n"/>
-      <c r="C93" s="3" t="n"/>
-      <c r="D93" s="3" t="n"/>
+      <c r="B93" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C93" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="E93" s="3" t="n"/>
       <c r="F93" s="2">
         <f>VLOOKUP($A93,Fixture!$A:$F,5,0)</f>
@@ -8072,9 +8104,17 @@
       <c r="A94" s="2" t="n">
         <v>93</v>
       </c>
-      <c r="B94" s="3" t="n"/>
-      <c r="C94" s="3" t="n"/>
-      <c r="D94" s="3" t="n"/>
+      <c r="B94" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C94" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="E94" s="3" t="n"/>
       <c r="F94" s="2">
         <f>VLOOKUP($A94,Fixture!$A:$F,5,0)</f>
@@ -8089,9 +8129,17 @@
       <c r="A95" s="2" t="n">
         <v>94</v>
       </c>
-      <c r="B95" s="3" t="n"/>
-      <c r="C95" s="3" t="n"/>
-      <c r="D95" s="3" t="n"/>
+      <c r="B95" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C95" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="E95" s="3" t="n"/>
       <c r="F95" s="2">
         <f>VLOOKUP($A95,Fixture!$A:$F,5,0)</f>
@@ -8106,9 +8154,17 @@
       <c r="A96" s="2" t="n">
         <v>95</v>
       </c>
-      <c r="B96" s="3" t="n"/>
-      <c r="C96" s="3" t="n"/>
-      <c r="D96" s="3" t="n"/>
+      <c r="B96" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C96" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
       <c r="E96" s="3" t="n"/>
       <c r="F96" s="2">
         <f>VLOOKUP($A96,Fixture!$A:$F,5,0)</f>

</xml_diff>

<commit_message>
chore: actualizar datos del torneo
</commit_message>
<xml_diff>
--- a/output/Mundial2026_Tracker.xlsx
+++ b/output/Mundial2026_Tracker.xlsx
@@ -5516,7 +5516,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>W96</t>
+          <t>Suiza</t>
         </is>
       </c>
       <c r="G101" s="2" t="n"/>
@@ -8179,17 +8179,27 @@
       <c r="A97" s="2" t="n">
         <v>96</v>
       </c>
-      <c r="B97" s="3" t="n"/>
-      <c r="C97" s="3" t="n"/>
-      <c r="D97" s="3" t="n"/>
-      <c r="E97" s="3" t="n"/>
-      <c r="F97" s="2">
-        <f>VLOOKUP($A97,Fixture!$A:$F,5,0)</f>
-        <v/>
-      </c>
-      <c r="G97" s="2">
-        <f>VLOOKUP($A97,Fixture!$A:$F,6,0)</f>
-        <v/>
+      <c r="B97" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C97" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>PEN</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Suiza</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G97" s="2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">

</xml_diff>